<commit_message>
Pipeline de modelagem atualizado e modelos ignorados no gitignore
</commit_message>
<xml_diff>
--- a/docs/DICIONÁRIO_DADOS_EXTERNOS.xlsx
+++ b/docs/DICIONÁRIO_DADOS_EXTERNOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aa2f146f46625b72/Área de Trabalho/TECH CHALLENGE 3/fiap_tech_challenge_03/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ademirasset.sharepoint.com/sites/TECNOLOGIA/Shared Documents/Geral/LUCAS/Estudos/FIAP/POSTECH_AI_SCIENTIST/tech_challenge_03/tech_challenge_03/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{1EB63BDE-B061-4F24-A4BC-B6F4820FA4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{370FF2AB-873D-4F8C-91B1-D8EAB060B3B2}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="8_{1EB63BDE-B061-4F24-A4BC-B6F4820FA4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33C40C82-9361-49BD-8835-B416C03CCB7D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D99BD419-5EC9-4AB4-B391-7B74A1983227}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{D99BD419-5EC9-4AB4-B391-7B74A1983227}"/>
   </bookViews>
   <sheets>
     <sheet name="fact_escola" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="128">
   <si>
     <t>ANO</t>
   </si>
@@ -413,6 +413,18 @@
   </si>
   <si>
     <t>Renda percapita média por estado</t>
+  </si>
+  <si>
+    <t>fact_uf_ano</t>
+  </si>
+  <si>
+    <t>fact_município</t>
+  </si>
+  <si>
+    <t>fact_escola</t>
+  </si>
+  <si>
+    <t>Tabela</t>
   </si>
 </sst>
 </file>
@@ -503,10 +515,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -827,145 +835,145 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86CCD61-D0EF-4322-AC51-D5FBF97B95A3}">
   <dimension ref="A1:U44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="81.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="81.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1"/>
     <col min="7" max="7" width="1" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.88671875" style="1"/>
+    <col min="8" max="9" width="8.85546875" style="1"/>
     <col min="10" max="10" width="1" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="1"/>
+    <col min="11" max="11" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="1"/>
     <col min="13" max="13" width="1" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" style="1"/>
+    <col min="14" max="14" width="6.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.85546875" style="1"/>
     <col min="16" max="16" width="1" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.88671875" style="1"/>
+    <col min="17" max="17" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" style="1"/>
     <col min="19" max="19" width="1" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="8.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.88671875" style="1"/>
-    <col min="22" max="22" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8.88671875" style="1"/>
-    <col min="25" max="25" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.88671875" style="1"/>
-    <col min="28" max="28" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="8.88671875" style="1"/>
-    <col min="31" max="31" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.88671875" style="1"/>
-    <col min="34" max="34" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="17.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.88671875" style="1"/>
-    <col min="37" max="37" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.88671875" style="1"/>
-    <col min="40" max="40" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.88671875" style="1"/>
-    <col min="43" max="43" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="10.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="8.88671875" style="1"/>
-    <col min="46" max="46" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="8.88671875" style="1"/>
-    <col min="49" max="49" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="8.88671875" style="1"/>
-    <col min="52" max="52" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="8.88671875" style="1"/>
-    <col min="55" max="55" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="8.88671875" style="1"/>
-    <col min="58" max="58" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="8.88671875" style="1"/>
-    <col min="61" max="61" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="8.88671875" style="1"/>
-    <col min="64" max="64" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="8.88671875" style="1"/>
-    <col min="67" max="67" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="8.88671875" style="1"/>
-    <col min="70" max="70" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="8.88671875" style="1"/>
-    <col min="73" max="73" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="8.88671875" style="1"/>
-    <col min="76" max="76" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="8.88671875" style="1"/>
-    <col min="79" max="79" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="8.88671875" style="1"/>
-    <col min="82" max="82" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="8.88671875" style="1"/>
-    <col min="85" max="85" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="8.88671875" style="1"/>
-    <col min="88" max="88" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="8.88671875" style="1"/>
-    <col min="91" max="91" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="8.88671875" style="1"/>
-    <col min="94" max="94" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="13.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="96" max="96" width="8.88671875" style="1"/>
-    <col min="97" max="97" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="8.85546875" style="1"/>
+    <col min="22" max="22" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.85546875" style="1"/>
+    <col min="25" max="25" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.85546875" style="1"/>
+    <col min="28" max="28" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8.85546875" style="1"/>
+    <col min="31" max="31" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.85546875" style="1"/>
+    <col min="34" max="34" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="8.85546875" style="1"/>
+    <col min="37" max="37" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="8.85546875" style="1"/>
+    <col min="40" max="40" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.85546875" style="1"/>
+    <col min="43" max="43" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="8.85546875" style="1"/>
+    <col min="46" max="46" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="8.85546875" style="1"/>
+    <col min="49" max="49" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="8.85546875" style="1"/>
+    <col min="52" max="52" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="8.85546875" style="1"/>
+    <col min="55" max="55" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="8.85546875" style="1"/>
+    <col min="58" max="58" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="8.85546875" style="1"/>
+    <col min="61" max="61" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="8.85546875" style="1"/>
+    <col min="64" max="64" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="8.85546875" style="1"/>
+    <col min="67" max="67" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="8.85546875" style="1"/>
+    <col min="70" max="70" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="8.85546875" style="1"/>
+    <col min="73" max="73" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="8.85546875" style="1"/>
+    <col min="76" max="76" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="8.85546875" style="1"/>
+    <col min="79" max="79" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="8.85546875" style="1"/>
+    <col min="82" max="82" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="8.85546875" style="1"/>
+    <col min="85" max="85" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="8.85546875" style="1"/>
+    <col min="88" max="88" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="8.85546875" style="1"/>
+    <col min="91" max="91" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="93" max="93" width="8.85546875" style="1"/>
+    <col min="94" max="94" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="96" max="96" width="8.85546875" style="1"/>
+    <col min="97" max="97" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="98" max="98" width="14" style="1" bestFit="1" customWidth="1"/>
-    <col min="99" max="99" width="8.88671875" style="1"/>
-    <col min="100" max="100" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="9.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="8.88671875" style="1"/>
-    <col min="103" max="103" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="18.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="105" max="105" width="8.88671875" style="1"/>
-    <col min="106" max="106" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="107" max="107" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="108" max="108" width="8.88671875" style="1"/>
-    <col min="109" max="109" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="110" max="110" width="25.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="111" max="111" width="8.88671875" style="1"/>
-    <col min="112" max="112" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="113" max="113" width="21.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="114" max="114" width="8.88671875" style="1"/>
-    <col min="115" max="115" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="116" max="116" width="22.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="8.88671875" style="1"/>
-    <col min="118" max="118" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="20.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="8.88671875" style="1"/>
-    <col min="121" max="121" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="8.88671875" style="1"/>
-    <col min="124" max="124" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="27.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="126" max="126" width="8.88671875" style="1"/>
-    <col min="127" max="127" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="99" max="99" width="8.85546875" style="1"/>
+    <col min="100" max="100" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="8.85546875" style="1"/>
+    <col min="103" max="103" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="104" max="104" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="105" max="105" width="8.85546875" style="1"/>
+    <col min="106" max="106" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="8.85546875" style="1"/>
+    <col min="109" max="109" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="110" max="110" width="25.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="111" max="111" width="8.85546875" style="1"/>
+    <col min="112" max="112" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="113" max="113" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="114" max="114" width="8.85546875" style="1"/>
+    <col min="115" max="115" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="8.85546875" style="1"/>
+    <col min="118" max="118" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="20.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="8.85546875" style="1"/>
+    <col min="121" max="121" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="18.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="8.85546875" style="1"/>
+    <col min="124" max="124" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="125" max="125" width="27.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="126" max="126" width="8.85546875" style="1"/>
+    <col min="127" max="127" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="128" max="128" width="36" style="1" bestFit="1" customWidth="1"/>
-    <col min="129" max="129" width="8.88671875" style="1"/>
-    <col min="130" max="130" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="131" max="131" width="34.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="132" max="132" width="8.88671875" style="1"/>
-    <col min="133" max="133" width="1.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="134" max="134" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="135" max="16384" width="8.88671875" style="1"/>
+    <col min="129" max="129" width="8.85546875" style="1"/>
+    <col min="130" max="130" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="131" max="131" width="34.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="132" max="132" width="8.85546875" style="1"/>
+    <col min="133" max="133" width="1.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="134" max="134" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="135" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>117</v>
       </c>
@@ -978,8 +986,11 @@
       <c r="D1" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E1" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -992,10 +1003,12 @@
       <c r="D2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="2"/>
+      <c r="E2" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1008,8 +1021,11 @@
       <c r="D3" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E3" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1022,8 +1038,11 @@
       <c r="D4" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E4" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1036,7 +1055,9 @@
       <c r="D5" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -1054,7 +1075,7 @@
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
     </row>
-    <row r="6" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1067,8 +1088,11 @@
       <c r="D6" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E6" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1081,8 +1105,11 @@
       <c r="D7" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E7" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1095,8 +1122,11 @@
       <c r="D8" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E8" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1109,8 +1139,11 @@
       <c r="D9" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E9" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1123,8 +1156,11 @@
       <c r="D10" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E10" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1137,8 +1173,11 @@
       <c r="D11" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E11" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>29</v>
       </c>
@@ -1151,8 +1190,11 @@
       <c r="D12" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E12" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>30</v>
       </c>
@@ -1165,8 +1207,11 @@
       <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E13" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>31</v>
       </c>
@@ -1179,8 +1224,11 @@
       <c r="D14" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E14" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
@@ -1193,8 +1241,11 @@
       <c r="D15" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E15" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>33</v>
       </c>
@@ -1207,8 +1258,11 @@
       <c r="D16" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E16" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -1221,8 +1275,11 @@
       <c r="D17" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E17" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -1235,8 +1292,11 @@
       <c r="D18" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E18" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
@@ -1249,8 +1309,11 @@
       <c r="D19" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E19" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
@@ -1263,8 +1326,11 @@
       <c r="D20" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E20" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>38</v>
       </c>
@@ -1277,8 +1343,11 @@
       <c r="D21" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E21" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>39</v>
       </c>
@@ -1291,8 +1360,11 @@
       <c r="D22" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E22" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>40</v>
       </c>
@@ -1305,8 +1377,11 @@
       <c r="D23" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E23" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>41</v>
       </c>
@@ -1319,8 +1394,11 @@
       <c r="D24" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E24" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>42</v>
       </c>
@@ -1333,8 +1411,11 @@
       <c r="D25" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E25" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>43</v>
       </c>
@@ -1347,8 +1428,11 @@
       <c r="D26" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E26" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>44</v>
       </c>
@@ -1361,8 +1445,11 @@
       <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E27" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>45</v>
       </c>
@@ -1375,8 +1462,11 @@
       <c r="D28" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E28" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>46</v>
       </c>
@@ -1389,8 +1479,11 @@
       <c r="D29" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E29" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>47</v>
       </c>
@@ -1403,8 +1496,11 @@
       <c r="D30" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E30" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>48</v>
       </c>
@@ -1417,8 +1513,11 @@
       <c r="D31" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E31" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>49</v>
       </c>
@@ -1431,8 +1530,11 @@
       <c r="D32" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E32" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>50</v>
       </c>
@@ -1445,8 +1547,11 @@
       <c r="D33" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E33" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>51</v>
       </c>
@@ -1459,8 +1564,11 @@
       <c r="D34" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E34" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1473,8 +1581,11 @@
       <c r="D35" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E35" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>11</v>
       </c>
@@ -1487,8 +1598,11 @@
       <c r="D36" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E36" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>12</v>
       </c>
@@ -1501,8 +1615,11 @@
       <c r="D37" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E37" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>13</v>
       </c>
@@ -1515,8 +1632,11 @@
       <c r="D38" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E38" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>14</v>
       </c>
@@ -1529,8 +1649,11 @@
       <c r="D39" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E39" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>15</v>
       </c>
@@ -1543,8 +1666,11 @@
       <c r="D40" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E40" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>16</v>
       </c>
@@ -1557,8 +1683,11 @@
       <c r="D41" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E41" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>17</v>
       </c>
@@ -1571,8 +1700,11 @@
       <c r="D42" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E42" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>18</v>
       </c>
@@ -1585,8 +1717,11 @@
       <c r="D43" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E43" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="49.5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>19</v>
       </c>
@@ -1598,6 +1733,9 @@
       </c>
       <c r="D44" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1608,17 +1746,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50E1EA0F-B798-4508-A51E-83A1D7D0CBFB}">
-  <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="81.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="16.28515625" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>117</v>
       </c>
@@ -1631,8 +1769,11 @@
       <c r="D1" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E1" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1645,8 +1786,11 @@
       <c r="D2" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1659,8 +1803,11 @@
       <c r="D3" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E3" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1673,8 +1820,11 @@
       <c r="D4" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1687,8 +1837,11 @@
       <c r="D5" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1701,8 +1854,11 @@
       <c r="D6" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E6" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1715,8 +1871,11 @@
       <c r="D7" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1729,8 +1888,11 @@
       <c r="D8" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1743,8 +1905,11 @@
       <c r="D9" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1757,8 +1922,11 @@
       <c r="D10" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>30</v>
       </c>
@@ -1771,8 +1939,11 @@
       <c r="D11" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -1785,8 +1956,11 @@
       <c r="D12" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>32</v>
       </c>
@@ -1799,8 +1973,11 @@
       <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>33</v>
       </c>
@@ -1813,8 +1990,11 @@
       <c r="D14" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>34</v>
       </c>
@@ -1827,8 +2007,11 @@
       <c r="D15" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E15" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>35</v>
       </c>
@@ -1841,8 +2024,11 @@
       <c r="D16" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>36</v>
       </c>
@@ -1855,8 +2041,11 @@
       <c r="D17" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E17" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>37</v>
       </c>
@@ -1869,8 +2058,11 @@
       <c r="D18" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
@@ -1883,8 +2075,11 @@
       <c r="D19" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>39</v>
       </c>
@@ -1897,8 +2092,11 @@
       <c r="D20" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>40</v>
       </c>
@@ -1911,8 +2109,11 @@
       <c r="D21" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>41</v>
       </c>
@@ -1925,8 +2126,11 @@
       <c r="D22" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1939,8 +2143,11 @@
       <c r="D23" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>43</v>
       </c>
@@ -1953,8 +2160,11 @@
       <c r="D24" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>44</v>
       </c>
@@ -1967,8 +2177,11 @@
       <c r="D25" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>45</v>
       </c>
@@ -1981,8 +2194,11 @@
       <c r="D26" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>46</v>
       </c>
@@ -1995,8 +2211,11 @@
       <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>47</v>
       </c>
@@ -2009,8 +2228,11 @@
       <c r="D28" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>48</v>
       </c>
@@ -2023,8 +2245,11 @@
       <c r="D29" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E29" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>49</v>
       </c>
@@ -2037,8 +2262,11 @@
       <c r="D30" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E30" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>66</v>
       </c>
@@ -2051,8 +2279,11 @@
       <c r="D31" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E31" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>67</v>
       </c>
@@ -2065,8 +2296,11 @@
       <c r="D32" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E32" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>68</v>
       </c>
@@ -2079,8 +2313,11 @@
       <c r="D33" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E33" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>69</v>
       </c>
@@ -2093,8 +2330,11 @@
       <c r="D34" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E34" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>70</v>
       </c>
@@ -2107,8 +2347,11 @@
       <c r="D35" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E35" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>71</v>
       </c>
@@ -2121,8 +2364,11 @@
       <c r="D36" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E36" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>15</v>
       </c>
@@ -2135,8 +2381,11 @@
       <c r="D37" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E37" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>16</v>
       </c>
@@ -2149,8 +2398,11 @@
       <c r="D38" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E38" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>17</v>
       </c>
@@ -2163,8 +2415,11 @@
       <c r="D39" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E39" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>18</v>
       </c>
@@ -2177,8 +2432,11 @@
       <c r="D40" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E40" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>19</v>
       </c>
@@ -2190,6 +2448,9 @@
       </c>
       <c r="D41" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2199,14 +2460,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABA1D795-6D60-4E0F-900C-3EF339D72D10}">
-  <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="52" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="103.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>117</v>
       </c>
@@ -2219,8 +2482,11 @@
       <c r="D1" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E1" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2233,8 +2499,11 @@
       <c r="D2" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -2247,8 +2516,11 @@
       <c r="D3" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2261,8 +2533,11 @@
       <c r="D4" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -2275,8 +2550,11 @@
       <c r="D5" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -2289,8 +2567,11 @@
       <c r="D6" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>77</v>
       </c>
@@ -2303,8 +2584,11 @@
       <c r="D7" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -2317,8 +2601,11 @@
       <c r="D8" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -2331,8 +2618,11 @@
       <c r="D9" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -2345,8 +2635,11 @@
       <c r="D10" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -2359,8 +2652,11 @@
       <c r="D11" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -2373,8 +2669,11 @@
       <c r="D12" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -2387,8 +2686,11 @@
       <c r="D13" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E13" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -2401,8 +2703,11 @@
       <c r="D14" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E14" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -2415,8 +2720,11 @@
       <c r="D15" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E15" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -2429,8 +2737,11 @@
       <c r="D16" s="2" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E16" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -2443,8 +2754,11 @@
       <c r="D17" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E17" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -2457,8 +2771,11 @@
       <c r="D18" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E18" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2471,8 +2788,11 @@
       <c r="D19" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E19" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -2485,8 +2805,11 @@
       <c r="D20" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E20" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -2499,8 +2822,11 @@
       <c r="D21" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E21" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -2513,8 +2839,11 @@
       <c r="D22" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E22" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -2527,8 +2856,11 @@
       <c r="D23" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E23" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -2541,8 +2873,11 @@
       <c r="D24" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>47</v>
       </c>
@@ -2555,8 +2890,11 @@
       <c r="D25" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E25" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>48</v>
       </c>
@@ -2569,8 +2907,11 @@
       <c r="D26" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E26" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -2583,8 +2924,11 @@
       <c r="D27" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E27" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>50</v>
       </c>
@@ -2597,8 +2941,11 @@
       <c r="D28" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>78</v>
       </c>
@@ -2611,8 +2958,11 @@
       <c r="D29" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E29" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>79</v>
       </c>
@@ -2625,8 +2975,11 @@
       <c r="D30" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E30" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>80</v>
       </c>
@@ -2639,8 +2992,11 @@
       <c r="D31" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E31" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>81</v>
       </c>
@@ -2653,8 +3009,11 @@
       <c r="D32" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>82</v>
       </c>
@@ -2667,16 +3026,281 @@
       <c r="D33" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="E33" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="33" x14ac:dyDescent="0.25">
       <c r="C34" s="1" t="s">
         <v>62</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="E34" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B2F5B2064B709C4B96B2BB6BA56010CA" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6e77452eb2d51676985a1637b279e587">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="242e9f65-b814-4ed0-b249-7801049d5c23" xmlns:ns3="051cde21-3992-497a-b8fe-9bb2eb9c95f5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5651a2f29d7f5045b92107f105f1c6b0" ns2:_="" ns3:_="">
+    <xsd:import namespace="242e9f65-b814-4ed0-b249-7801049d5c23"/>
+    <xsd:import namespace="051cde21-3992-497a-b8fe-9bb2eb9c95f5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="242e9f65-b814-4ed0-b249-7801049d5c23" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="394d2bc3-e22e-42db-b4dd-8ec92871baac" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="051cde21-3992-497a-b8fe-9bb2eb9c95f5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{2b48e568-db8f-49b3-a172-8970c3cec87e}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="051cde21-3992-497a-b8fe-9bb2eb9c95f5">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="242e9f65-b814-4ed0-b249-7801049d5c23">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="051cde21-3992-497a-b8fe-9bb2eb9c95f5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67245022-79CD-4A50-BFED-6B4D47EEC452}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="242e9f65-b814-4ed0-b249-7801049d5c23"/>
+    <ds:schemaRef ds:uri="051cde21-3992-497a-b8fe-9bb2eb9c95f5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E092E88-C537-4C47-9A5D-7F336B708525}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F89A9DF-7BAB-4880-BDA0-576D8D6D22F4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="242e9f65-b814-4ed0-b249-7801049d5c23"/>
+    <ds:schemaRef ds:uri="051cde21-3992-497a-b8fe-9bb2eb9c95f5"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>